<commit_message>
[Arif Iqubal] : udated Testplan and testdata document
</commit_message>
<xml_diff>
--- a/06_Test_Data/TestData.xlsx
+++ b/06_Test_Data/TestData.xlsx
@@ -7,7 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LoginData" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RegistrationData" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductData" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CheckoutData" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,23 +416,383 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>TestCaseID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Email</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Password</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ExpectedResult</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TC001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>validuser@test.com</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ValidPass123</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Login Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TC002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>validuser@test.com</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>WrongPass</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Error Message</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TC003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>wronguser@test.com</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ValidPass123</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Error Message</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TC004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Validation Message</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TestCaseID</t>
+        </is>
+      </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Password</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ExpectedResult</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TC006</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>john123@test.com</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>John@123</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Registration Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TC007</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Jane Smith</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>john123@test.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Jane@123</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Error Existing Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TC008</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Validation Message</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TestCaseID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ProductName</t>
+        </is>
+      </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>ProductName</t>
+          <t>ExpectedResult</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TC011</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Blue Top</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Product Added</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TC012</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Men Tshirt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Product Added</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TC013</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Sleeveless Dress</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Product Removed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TestCaseID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ExpectedResult</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TC016</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Street 1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Checkout Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TC017</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Validation Message</t>
         </is>
       </c>
     </row>

</xml_diff>